<commit_message>
Weekly results: Phil 02-23, Vivienne 02-23/02-28, Rosalind 03-02
- Master databases updated
- Delivery emails generated
- Funding intel CSVs
</commit_message>
<xml_diff>
--- a/results/For_Others/Phil_Tassi/Week_of_2026-02-23/deliverables/Phil_Tassi_Master_List_2026-02-23.xlsx
+++ b/results/For_Others/Phil_Tassi/Week_of_2026-02-23/deliverables/Phil_Tassi_Master_List_2026-02-23.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Search Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$5:$N$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Search Results'!$A$5:$N$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -67,7 +67,7 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="00595959"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -137,9 +137,15 @@
   </cellStyleXfs>
   <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -170,10 +176,10 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -542,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -561,27 +567,28 @@
     <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Phil Tassi — Master Job List</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Week of February 23, 2026  |  Prepared by Joey Clark</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>37 jobs  |  Score range: 70-93  |  Avg: 79.4  |  13 NEW, 24 REPEAT</t>
-        </is>
-      </c>
-    </row>
+          <t>47 jobs  |  Score range: 70-93  |  Avg: 79  |  10 NEW, 37 REPEAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="10" customHeight="1"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -660,12 +667,14 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
-        <v>93</v>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Perfect intersection of commercial banking expertise and partnership development. Business banking focus directly matches JPMorgan startup banking experience (40/40 skills, 35/35 industry, 18/25 experience).</t>
+          <t>Perfect intersection of commercial banking expertise and partnership development. Business banking focus directly matches JPMorgan startup banking experience. (40/40 skills, 35/35 industry, 18/25 experience).</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -700,12 +709,12 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>£105,000-£130,000 + equity</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Drive ambitious growth targets for Monzo Business Banking through strategic partnerships. First Business Banking Growth Partnerships Lead role, focused on the switcher market.</t>
+          <t>First Business Banking Growth Partnerships Lead. Drive ambitious growth targets; 1 in 6 new businesses apply for Monzo Business account. Pivotal role identifying strategic partnerships.</t>
         </is>
       </c>
       <c r="L6" s="8" t="inlineStr">
@@ -730,8 +739,10 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>92</v>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
@@ -800,27 +811,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
-        <v>90</v>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Strong zero-to-one fit at financial automation startup. CoS role matches operator background perfectly. Financial sector aligns with JPMorgan/SVB experience (38/40 skills, 30/35 industry, 22/25 experience).</t>
+          <t>Premier fintech unicorn CoS-to-CEO role. IPO readiness leverages finance/strategy MBA. Payments sector directly aligns (40/40 skills, 35/35 industry, 16/25 experience).</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>LiveFlow</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Chief of Staff</t>
+          <t>Chief of Staff - CEO</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Fintech/Financial Automation</t>
+          <t>Fintech/Payments</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -845,12 +858,12 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Chief of Staff at financial automation startup. Partner with CEO on strategic initiatives, cross-functional execution, and company-building at early stage.</t>
+          <t>Premier fintech unicorn CoS-to-CEO role. IPO readiness work leverages finance/strategy MBA.</t>
         </is>
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/liveflow/df3eb756-fcb2-4a0a-adff-1556c28b919a</t>
+          <t>https://jobs.ashbyhq.com/airwallex/26923274-95b8-4365-b8ab-fa09e6755004</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -870,104 +883,108 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
-        <v>88</v>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Direct fintech/banking alignment at UK's leading neobank. CEO-level CoS matches operator background perfectly. 10+ years experience requirement is a stretch but VP experience is strong (36/40 skills, 35/35 industry, 17/25 experience).</t>
+          <t>Phil has direct Techstars experience. Strategy &amp; ops CoS to CEO matches perfectly. VC/accelerator sector directly relevant. 2-3 year rotational structure is ideal (40/40 skills, 30/35 industry, 20/25 experience).</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Monzo</t>
+          <t>Techstars</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Chief of Staff (CEO)</t>
+          <t>Chief of Staff</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Fintech/Banking</t>
+          <t>Venture Capital/Accelerators</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
+          <t>US East Coast</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>Strategy and operations-minded CoS working closely with CEO. 2-3 year assignment to build deep understanding then lead a business area.</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/techstars57/jobs/5451541002</t>
+        </is>
+      </c>
+      <c r="M9" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N9" s="11" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Strong zero-to-one fit at financial automation startup. CoS matches operator background perfectly (38/40 skills, 30/35 industry, 22/25 experience).</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>LiveFlow</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Chief of Staff</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Fintech/Financial Automation</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
           <t>London</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K9" s="10" t="inlineStr">
-        <is>
-          <t>Chief of Staff to CEO at UK's leading digital bank. Drive critical strategic projects and own cross-functional initiatives. Report directly to CEO with board exposure.</t>
-        </is>
-      </c>
-      <c r="L9" s="11" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/monzo/jobs/2289088</t>
-        </is>
-      </c>
-      <c r="M9" s="11" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N9" s="11" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="n">
-        <v>87</v>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Fintech infrastructure partnerships at Plaid. GTM partnerships team unlocks 'one to many' customer relationships. Fintech sector is a perfect match. London office available (36/40 skills, 35/35 industry, 16/25 experience).</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Plaid</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Partnerships Account Executive - Enterprise</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Fintech/Payments Infrastructure</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -985,12 +1002,12 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>GTM Partnerships team role unlocking one-to-many customer relationships with technology platforms. Plaid offices in San Francisco, New York, Washington DC, London, and Amsterdam.</t>
+          <t>Chief of Staff at financial automation startup. Partner with CEO on strategic initiatives.</t>
         </is>
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/plaid/b134ba8a-eac5-4271-a279-3ed0176b24de</t>
+          <t>https://jobs.ashbyhq.com/liveflow/df3eb756-fcb2-4a0a-adff-1556c28b919a</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -1000,7 +1017,7 @@
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>Lever</t>
+          <t>Ashby</t>
         </is>
       </c>
     </row>
@@ -1010,27 +1027,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n">
-        <v>86</v>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Fintech CoS role aligns with commercial operator expertise. Early-stage company matches zero-to-one build experience from JPMorgan LA (36/40 skills, 30/35 industry, 20/25 experience).</t>
+          <t>Direct fintech sector alignment at UK's leading neobank. CEO-level CoS matches operator background perfectly. 10+ years requirement aligns with VP seniority (36/40 skills, 35/35 industry, 17/25 experience).</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Tilt</t>
+          <t>Monzo</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Chief of Staff</t>
+          <t>Chief of Staff (CEO)</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Fintech/Corporate Cards</t>
+          <t>Fintech/Banking</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -1055,12 +1074,12 @@
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
-          <t>Chief of Staff at early-stage fintech corporate cards company. Partner with CEO on strategy, operations, and company-building. Zero-to-one build opportunity.</t>
+          <t>Chief of Staff to CEO at UK's leading digital bank. At the centre of Monzo working with leadership team to deliver critical projects. Requires 10+ years experience.</t>
         </is>
       </c>
       <c r="L11" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/tilt/fe2c6309-3dfc-4fd5-9e32-854fe09a0bc0</t>
+          <t>https://boards.greenhouse.io/monzo/jobs/2289088</t>
         </is>
       </c>
       <c r="M11" s="11" t="inlineStr">
@@ -1070,7 +1089,7 @@
       </c>
       <c r="N11" s="11" t="inlineStr">
         <is>
-          <t>Ashby</t>
+          <t>Greenhouse</t>
         </is>
       </c>
     </row>
@@ -1080,27 +1099,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n">
-        <v>85</v>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Cross-functional strategic execution aligns well with JPMorgan experience and operator background. Tech/marketplace sector less fintech-aligned but company scale and CEO-reporting structure is excellent (36/40 skills, 22/35 industry, 27/25 experience - capped at 25).</t>
+          <t>Enterprise BD with C-suite negotiations directly matches Phil's experience. 6-10 years payments/fintech requirement aligns. Crypto/payments sector adjacent to banking (38/40 skills, 28/35 industry, 22/25 experience).</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Deliveroo</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Chief of Staff to CEO</t>
+          <t>Business Partnership Manager - Payment</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Food Tech/Marketplace</t>
+          <t>Crypto/Payments</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -1125,12 +1146,12 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Support CEO and Executive team with operational support, mission-critical projects, and strategic initiatives. Highly cross-functional role with broad exposure across every dimension of the business.</t>
+          <t>6-10 years payments/fintech experience. Enterprise-level BD engaging C-suite stakeholders.</t>
         </is>
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/deliveroo/jobs/4164199</t>
+          <t>https://jobs.lever.co/binance/ebd6b52e-c402-49f9-8945-88a7f6e4cd60</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -1140,7 +1161,7 @@
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>Lever</t>
         </is>
       </c>
     </row>
@@ -1150,104 +1171,108 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
-        <v>84</v>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Chief of Staff at green fintech bank. Direct fintech sector alignment and CEO-reporting structure matches operator profile well. Sustainable finance is growth sector (36/40 skills, 35/35 industry, 13/25 experience).</t>
+          <t>Director-level fintech partnerships at leading corporate card company. Directly matches BD/partnerships expertise (40/40 skills, 35/35 industry, 13/25 experience).</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Tandem Bank</t>
+          <t>Ramp</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Chief of Staff</t>
+          <t>Director - Product Partnerships</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Fintech/Banking</t>
+          <t>Fintech/Corporate Cards</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>$255,000-$300,000</t>
+        </is>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>Director-level fintech partnerships at leading corporate card company.</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/ramp/224449f1-5164-41af-8c5b-d3cb33cf6621</t>
+        </is>
+      </c>
+      <c r="M13" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N13" s="11" t="inlineStr">
+        <is>
+          <t>Ashby</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Fintech infrastructure partnerships at Plaid. GTM partnerships unlock one-to-many customer relationships. Fintech sector perfect match (36/40 skills, 35/35 industry, 16/25 experience).</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Plaid</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Partnerships Account Executive - Enterprise</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Fintech/Payments Infrastructure</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
           <t>London</t>
         </is>
       </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I13" s="11" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J13" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
-        <is>
-          <t>Report to CEO working across all aspects of cross-functional projects. UK's greener digital bank with £1.5bn in assets under management, focused on sustainable finance.</t>
-        </is>
-      </c>
-      <c r="L13" s="11" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/tandemmoneylimited/jobs/6206792002</t>
-        </is>
-      </c>
-      <c r="M13" s="11" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N13" s="11" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="n">
-        <v>84</v>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>First Revenue Partnerships hire at leading AI voice company. Builder role perfectly matches zero-to-one experience. AI sector is high-growth. London office available (36/40 skills, 28/35 industry, 20/25 experience).</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>ElevenLabs</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Revenue Partnerships</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>AI/Voice Tech</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -1255,7 +1280,7 @@
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Remote-Global</t>
+          <t>Hybrid</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr">
@@ -1265,12 +1290,12 @@
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>First Revenue Partnerships hire at ElevenLabs, the leading AI voice technology company. Build partnerships function from scratch. Optional offices in London, New York, San Francisco.</t>
+          <t>GTM Partnerships team unlocking one-to-many customer relationships with technology platforms.</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/elevenlabs/708b7152-f22a-4531-94a9-0f91cc0c1a70</t>
+          <t>https://jobs.lever.co/plaid/b134ba8a-eac5-4271-a279-3ed0176b24de</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -1280,7 +1305,7 @@
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>Ashby</t>
+          <t>Lever</t>
         </is>
       </c>
     </row>
@@ -1290,32 +1315,34 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
-        <v>83</v>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Phil's VC background uniquely qualifies for VC partnership development. HR Tech/fintech adjacent sector. Remote-global works for London base (38/40 skills, 25/35 industry, 20/25 experience).</t>
+          <t>Fintech CoS aligns with commercial operator expertise. Early-stage matches zero-to-one experience (36/40 skills, 30/35 industry, 20/25 experience).</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Deel</t>
+          <t>Tilt</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Partnerships Manager - Venture Capital</t>
+          <t>Chief of Staff</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>HR Tech/Fintech</t>
+          <t>Fintech/Corporate Cards</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
@@ -1325,7 +1352,7 @@
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>Remote-Global</t>
+          <t>Hybrid</t>
         </is>
       </c>
       <c r="J15" s="11" t="inlineStr">
@@ -1335,12 +1362,12 @@
       </c>
       <c r="K15" s="10" t="inlineStr">
         <is>
-          <t>Lead venture capital partnerships at Deel, the global HR and payroll platform. Leverage VC network to drive strategic partnerships and ecosystem growth.</t>
+          <t>Chief of Staff at early-stage fintech corporate cards company.</t>
         </is>
       </c>
       <c r="L15" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/deel/90aefa1d-30b5-4b43-82c2-53348fbc64b9</t>
+          <t>https://jobs.ashbyhq.com/tilt/fe2c6309-3dfc-4fd5-9e32-854fe09a0bc0</t>
         </is>
       </c>
       <c r="M15" s="11" t="inlineStr">
@@ -1360,27 +1387,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n">
-        <v>83</v>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Chief of Staff EMEA at global communications platform. Cross-functional strategic execution and partnership skills transfer well. EMEA scope matches London base (38/40 skills, 28/35 industry, 17/25 experience).</t>
+          <t>Cross-functional strategic execution aligns with JPMorgan experience. Marketplace tech less fintech-aligned but company scale and CEO-reporting structure is excellent (36/40 skills, 22/35 industry, 25/25 experience).</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Deliveroo</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Chief of Staff EMEA</t>
+          <t>Chief of Staff to the CEO</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Communications Tech</t>
+          <t>Food Tech/Marketplace</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
@@ -1405,12 +1434,12 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>Strategic and operational partner to EMEA leadership at Twilio. Drive mission-critical projects and cross-functional work. Hybrid role in Soho, London.</t>
+          <t>Support CEO and Executive team with operational support, mission-critical projects. Highly cross-functional with broad exposure across every dimension of the business.</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/twilio/jobs/3786401</t>
+          <t>https://boards.greenhouse.io/deliveroo/jobs/4164199</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -1430,17 +1459,19 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
-        <v>82</v>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Phil's VC background is directly relevant. Zero-to-one build at angel network matches startup banking experience. Small team = high impact (38/40 skills, 28/35 industry, 16/25 experience).</t>
+          <t>Direct fintech sector alignment at green digital bank. CEO-reporting structure matches operator profile. Sustainable finance is growth sector (36/40 skills, 35/35 industry, 13/25 experience).</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>CVX Ventures</t>
+          <t>Tandem Bank</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -1450,7 +1481,7 @@
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Venture Capital</t>
+          <t>Fintech/Banking</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -1475,12 +1506,12 @@
       </c>
       <c r="K17" s="10" t="inlineStr">
         <is>
-          <t>Lead CVX Ventures through next phase of expansion, driving the mission to build Europe's largest and most active angel investor network. Team across Copenhagen, London, Oslo.</t>
+          <t>Report to CEO across all aspects of cross-functional projects. UK's greener digital bank with £1.5bn in AUM, focused on sustainable finance and net-zero.</t>
         </is>
       </c>
       <c r="L17" s="11" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/cvx/jobs/6600987003</t>
+          <t>https://boards.greenhouse.io/tandemmoneylimited/jobs/6206792002</t>
         </is>
       </c>
       <c r="M17" s="11" t="inlineStr">
@@ -1500,27 +1531,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n">
-        <v>82</v>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Operational Director/Chief of Staff at fintech trading platform. Director-level role matches VP seniority in CoS context. Fintech/trading sector fully aligns (36/40 skills, 35/35 industry, 11/25 experience).</t>
+          <t>Build and scale strategic partnerships at world's leading AI company (36/40 skills, 28/35 industry, 20/25 experience).</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Capital.com</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Operational Director / Chief of Staff</t>
+          <t>Strategic Partnerships</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Fintech/Trading</t>
+          <t>AI/Technology</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
@@ -1545,12 +1578,12 @@
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>Strategic and operational partner to CIO/CISO. Translate organizational goals into execution plans with effective structures, resource planning, and consistent delivery.</t>
+          <t>Strategic Partnerships role at OpenAI. Build and scale partnerships at the world's leading AI company.</t>
         </is>
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/capital/a9d8380f-d02b-4e38-aa3a-fa895b94d125</t>
+          <t>https://jobs.ashbyhq.com/openai/aa881d4a-e8a9-4863-92b6-b64938bf88ed</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -1560,147 +1593,151 @@
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
+          <t>Ashby</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Cross-functional strategic execution and partnership skills transfer well. EMEA scope matches London base. Soho Square office (38/40 skills, 28/35 industry, 17/25 experience).</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Twilio</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Chief of Staff EMEA</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Communications Tech</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>Strategic and operational partner to EMEA leadership at Twilio. Hybrid role in Soho Square, London.</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/twilio/jobs/3786401</t>
+        </is>
+      </c>
+      <c r="M19" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N19" s="11" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>BD in payments/fintech matches commercial background. 5+ years required aligns (35/40 skills, 28/35 industry, 20/25 experience).</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Business Development - Payment</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Crypto/Payments</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>5+ years payments/fintech experience. Identify and onboard key merchants, PSPs, and strategic partners.</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/binance/722d8df0-09d5-47c5-b7d8-db9df02dfd8b</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N20" s="8" t="inlineStr">
+        <is>
           <t>Lever</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="n">
-        <v>82</v>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>Insurtech/fintech platform CoS role. High-trust role directly with CEO driving alignment and execution. Fintech-adjacent sector strongly aligns (34/40 skills, 28/35 industry, 20/25 experience).</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>Bjak</t>
-        </is>
-      </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>Chief of Staff - UK</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>Insurtech/Fintech</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K19" s="10" t="inlineStr">
-        <is>
-          <t>High-trust, high-leverage role working directly with the CEO to drive alignment, clarity, and execution across the organisation. Bjak builds superior application platforms globally.</t>
-        </is>
-      </c>
-      <c r="L19" s="11" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/bjakcareer/0fda5dff-ed04-4e75-a6bc-939535751cf8</t>
-        </is>
-      </c>
-      <c r="M19" s="11" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N19" s="11" t="inlineStr">
-        <is>
-          <t>Ashby</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n">
-        <v>82</v>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Fintech AI financial assistant CoS role. Direct fintech sector alignment. Leadership team coordination matches operator profile. Hybrid London works well (32/40 skills, 30/35 industry, 20/25 experience).</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Cleo</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Chief of Staff</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Fintech/AI</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I20" s="8" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K20" s="7" t="inlineStr">
-        <is>
-          <t>Bring the leadership team together and run team meetings in lieu of the CEO. Cleo is an AI-powered financial assistant. Hybrid-first role, London office 1-2 times a week.</t>
-        </is>
-      </c>
-      <c r="L20" s="8" t="inlineStr">
-        <is>
-          <t>https://uk.linkedin.com/jobs/view/chief-of-staff-at-cleo-3772186729</t>
-        </is>
-      </c>
-      <c r="M20" s="8" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N20" s="8" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
         </is>
       </c>
     </row>
@@ -1710,17 +1747,19 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B21" s="12" t="n">
-        <v>81</v>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Chief of Staff at financial services fintech. Strong fintech sector alignment and CEO-reporting structure matches operator profile (36/40 skills, 35/35 industry, 10/25 experience).</t>
+          <t>Phil's VC background directly relevant. Zero-to-one build at angel network matches startup banking. Small team = high impact (38/40 skills, 28/35 industry, 16/25 experience).</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Liberis</t>
+          <t>CVX Ventures</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -1730,7 +1769,7 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>Fintech/Financial Services</t>
+          <t>Venture Capital</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
@@ -1755,12 +1794,12 @@
       </c>
       <c r="K21" s="10" t="inlineStr">
         <is>
-          <t>Chief of Staff at Liberis, leading global provider of embedded business finance. Delivered more than £500M in funding to SMEs across UK, EU, and US.</t>
+          <t>Lead CVX Ventures through next expansion phase. Build Europe's largest angel investor network.</t>
         </is>
       </c>
       <c r="L21" s="11" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/liberis/jobs/3084965</t>
+          <t>https://job-boards.greenhouse.io/cvx/jobs/6690261003</t>
         </is>
       </c>
       <c r="M21" s="11" t="inlineStr">
@@ -1780,27 +1819,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n">
-        <v>81</v>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Payments fintech aligns with banking and fintech background. Partnership acquisition role directly matches BD/partnership expertise. UK &amp; FR scope is manageable (35/40 skills, 32/35 industry, 14/25 experience).</t>
+          <t>Operational Director/CoS at fintech trading platform. Director-level matches VP seniority (36/40 skills, 35/35 industry, 11/25 experience).</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Mollie</t>
+          <t>Capital.com</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Technology Partnerships Acquisition Manager - UK &amp; FR</t>
+          <t>Operational Director / Chief of Staff</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>Fintech/Payments</t>
+          <t>Fintech/Trading</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -1825,12 +1866,12 @@
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>Acquire and develop technology partnerships at Mollie, one of Europe's fastest-growing payment service providers. Focus on UK and France markets.</t>
+          <t>Strategic and operational partner to CIO/CISO. Translate goals into clear execution plans.</t>
         </is>
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/mollie/0141f0ed-59a1-4b32-b985-3c42fa6b64ac</t>
+          <t>https://jobs.lever.co/capital/a9d8380f-d02b-4e38-aa3a-fa895b94d125</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
@@ -1840,7 +1881,7 @@
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
-          <t>Ashby</t>
+          <t>Lever</t>
         </is>
       </c>
     </row>
@@ -1850,32 +1891,34 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B23" s="12" t="n">
-        <v>80</v>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>CEO-reporting CoS structure matches operator profile. DC hybrid location is a strong fit. AI/disinformation sector is growing (32/40 skills, 22/35 industry, 26/25 - capped at 25).</t>
+          <t>Insurtech/fintech platform CoS. High-trust role directly with CEO (34/40 skills, 28/35 industry, 20/25 experience).</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Alethea</t>
+          <t>Bjak</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Chief of Staff</t>
+          <t>Chief of Staff - UK</t>
         </is>
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>AI/Disinformation</t>
+          <t>Insurtech/Fintech</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>Washington DC</t>
+          <t>London</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
@@ -1895,12 +1938,12 @@
       </c>
       <c r="K23" s="10" t="inlineStr">
         <is>
-          <t>Collaborate with CEO and COO to drive initiatives, manage meetings, draft communications, prepare board materials. NYC or DC hybrid 3 days/week.</t>
+          <t>High-trust, high-leverage role working directly with CEO to drive alignment and execution.</t>
         </is>
       </c>
       <c r="L23" s="11" t="inlineStr">
         <is>
-          <t>https://boards.greenhouse.io/alethea/jobs/5050878004</t>
+          <t>https://jobs.ashbyhq.com/bjakcareer/0fda5dff-ed04-4e75-a6bc-939535751cf8</t>
         </is>
       </c>
       <c r="M23" s="11" t="inlineStr">
@@ -1910,7 +1953,7 @@
       </c>
       <c r="N23" s="11" t="inlineStr">
         <is>
-          <t>Greenhouse</t>
+          <t>Ashby</t>
         </is>
       </c>
     </row>
@@ -1920,27 +1963,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B24" s="12" t="n">
-        <v>80</v>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>GTM-focused CoS at well-funded startup matches zero-to-one execution background. SaaS/procurement sector less aligned but fintech client base is relevant (34/40 skills, 22/35 industry, 24/25 experience).</t>
+          <t>Payments fintech partnerships. UK &amp; FR scope manageable (35/40 skills, 32/35 industry, 14/25 experience).</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Omnea</t>
+          <t>Mollie</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Interim Chief of Staff - GTM</t>
+          <t>Technology Partnerships Acquisition Manager - UK &amp; FR</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>SaaS/Procurement</t>
+          <t>Fintech/Payments</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
@@ -1965,12 +2010,12 @@
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>Interim Chief of Staff, GTM at Omnea. Drive go-to-market strategy and execution at well-funded SaaS procurement platform with fintech client base.</t>
+          <t>Acquire and develop technology partnerships at Mollie, one of Europe's fastest-growing PSPs.</t>
         </is>
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/omnea/a81f0554-841c-45f2-8142-ddddab228793</t>
+          <t>https://jobs.ashbyhq.com/mollie/0141f0ed-59a1-4b32-b985-3c42fa6b64ac</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
@@ -1985,37 +2030,39 @@
       </c>
     </row>
     <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="14" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="n">
-        <v>80</v>
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Senior partnerships leader for EMEA at e-commerce platform. Director-level role matches VP seniority. Strategy and execution for high-impact partner relationships (38/40 skills, 20/35 industry, 22/25 experience).</t>
+          <t>CEO-reporting CoS matches operator profile. DC hybrid location strong fit. AI/disinformation sector growing (32/40 skills, 22/35 industry, 25/25 experience).</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Alethea</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>Director of Partnerships - EMEA</t>
+          <t>Chief of Staff</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>E-commerce Tech</t>
+          <t>AI/Disinformation</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Washington DC</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
@@ -2035,12 +2082,12 @@
       </c>
       <c r="K25" s="10" t="inlineStr">
         <is>
-          <t>Accelerate presence and pipeline across Europe through high-impact partner relationships. Lead strategy and execution for partnerships in EMEA. London office-based.</t>
+          <t>Individual contributor CoS collaborating with CEO and COO. Hybrid 3 days/week in DC or NYC office.</t>
         </is>
       </c>
       <c r="L25" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/pattern/fc621c26-c2ef-40bf-9fb4-3fee3d341436</t>
+          <t>https://boards.greenhouse.io/alethea/jobs/5050878004</t>
         </is>
       </c>
       <c r="M25" s="11" t="inlineStr">
@@ -2050,7 +2097,7 @@
       </c>
       <c r="N25" s="11" t="inlineStr">
         <is>
-          <t>Lever</t>
+          <t>Greenhouse</t>
         </is>
       </c>
     </row>
@@ -2060,27 +2107,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B26" s="15" t="n">
-        <v>78</v>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Phil's VC background uniquely qualifies for VC partnership development. Security SaaS industry is less aligned (38/40 skills, 18/35 industry, 22/25 experience).</t>
+          <t>Senior partnerships leader for EMEA. Director-level matches VP seniority (38/40 skills, 20/35 industry, 22/25 experience).</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Vanta</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>Strategic Venture Capital Partnerships Manager</t>
+          <t>Director of Partnerships - EMEA</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>Security/SaaS</t>
+          <t>E-commerce Tech</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -2105,12 +2154,12 @@
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>Founding member of Vanta's Venture &amp; Startup Partnerships team in EMEA. Build and scale presence across the London startup and VC ecosystem.</t>
+          <t>Senior partnerships leader for EMEA. Lead strategy and execution for partnerships to accelerate presence.</t>
         </is>
       </c>
       <c r="L26" s="8" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/vanta/4e32f84c-84c5-45a6-a8b5-2b3f71235286</t>
+          <t>https://jobs.lever.co/pattern/fc621c26-c2ef-40bf-9fb4-3fee3d341436</t>
         </is>
       </c>
       <c r="M26" s="8" t="inlineStr">
@@ -2120,37 +2169,39 @@
       </c>
       <c r="N26" s="8" t="inlineStr">
         <is>
-          <t>Ashby</t>
+          <t>Lever</t>
         </is>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="n">
-        <v>78</v>
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>CEO's core partner in ensuring organisational clarity, discipline and focus. Legal tech sector is adjacent to fintech. Strong compensation range (36/40 skills, 20/35 industry, 22/25 experience).</t>
+          <t>GTM-focused CoS at well-funded startup matches zero-to-one execution background (34/40 skills, 22/35 industry, 24/25 experience).</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Lawhive</t>
+          <t>Omnea</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>Chief of Staff to CEO</t>
+          <t>Interim Chief of Staff - GTM</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>Legal Tech</t>
+          <t>SaaS/Procurement</t>
         </is>
       </c>
       <c r="G27" s="11" t="inlineStr">
@@ -2170,17 +2221,17 @@
       </c>
       <c r="J27" s="11" t="inlineStr">
         <is>
-          <t>£110,000-£160,000 + options</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K27" s="10" t="inlineStr">
         <is>
-          <t>CEO's core partner ensuring the organisation runs with clarity, discipline and focus. London/Hybrid 3 days per week on-site. Series A legal tech startup.</t>
+          <t>Interim Chief of Staff, GTM. Drive go-to-market strategy and execution.</t>
         </is>
       </c>
       <c r="L27" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/lawhive/d579d249-abef-4972-8c6c-63be5af18b34</t>
+          <t>https://jobs.ashbyhq.com/omnea/a81f0554-841c-45f2-8142-ddddab228793</t>
         </is>
       </c>
       <c r="M27" s="11" t="inlineStr">
@@ -2200,27 +2251,29 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="B28" s="15" t="n">
-        <v>78</v>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Build partnerships with news publishing partners at leading AI company. Strong sector with high growth. EMEA scope matches London base (32/40 skills, 28/35 industry, 18/25 experience).</t>
+          <t>CoS Product at leading neobank. Product strategy focus with massive scope. Fintech sector perfect (26/40 skills, 35/35 industry, 17/25 experience).</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Monzo</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Partner Manager - News EMEA</t>
+          <t>Chief of Staff, Product</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>AI/Technology</t>
+          <t>Fintech/Banking</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
@@ -2245,12 +2298,12 @@
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>Build and nurture relationships with news publishing partners through 1:1 interactions, industry programs, and other partnerships at OpenAI. EMEA focus.</t>
+          <t>Chief of Staff, Product at Monzo. Lead product strategy with massive scope at the UK's leading digital bank.</t>
         </is>
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/openai/77a2ec4a-10ee-4c7e-b05f-881348b9b41f</t>
+          <t>https://boards.greenhouse.io/monzo/jobs/4589197</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
@@ -2260,254 +2313,262 @@
       </c>
       <c r="N28" s="8" t="inlineStr">
         <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>CoS to CEO at legaltech matches operator profile. £110-160K excellent comp. AI-first company is modern (36/40 skills, 20/35 industry, 22/25 experience).</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Lawhive</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>Chief of Staff to the CEO</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>LegalTech/AI</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I29" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J29" s="11" t="inlineStr">
+        <is>
+          <t>£110,000-£160,000 + share options</t>
+        </is>
+      </c>
+      <c r="K29" s="10" t="inlineStr">
+        <is>
+          <t>CEO's core partner ensuring organisation runs with clarity, discipline and focus. AI operating system reinventing legal industry. 3 days/week on-site.</t>
+        </is>
+      </c>
+      <c r="L29" s="11" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/lawhive/d579d249-abef-4972-8c6c-63be5af18b34</t>
+        </is>
+      </c>
+      <c r="M29" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N29" s="11" t="inlineStr">
+        <is>
           <t>Ashby</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="45" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="B29" s="15" t="n">
-        <v>78</v>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Partnerships sales at leading fintech. Broker/white-label models align with banking experience. Fintech/payments sector is excellent fit (32/40 skills, 32/35 industry, 14/25 experience).</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>Ebury</t>
-        </is>
-      </c>
-      <c r="E29" s="11" t="inlineStr">
-        <is>
-          <t>Sales Executive - Partnerships</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="inlineStr">
-        <is>
-          <t>Fintech/Payments</t>
-        </is>
-      </c>
-      <c r="G29" s="11" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>VC partnerships matches Phil's VC background. Founding EMEA role. Security/compliance SaaS growing (36/40 skills, 22/35 industry, 20/25 experience).</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Vanta</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Strategic Venture Capital Partnerships Manager</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Security/Compliance SaaS</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I29" s="11" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J29" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K29" s="10" t="inlineStr">
-        <is>
-          <t>Expand Partnerships Sales Team managing partners through introductory broker agreements and white-label solutions. Ebury has 1,700+ staff across 25+ countries worldwide.</t>
-        </is>
-      </c>
-      <c r="L29" s="11" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/ebury/jobs/4598559101</t>
-        </is>
-      </c>
-      <c r="M29" s="11" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N29" s="11" t="inlineStr">
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J30" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t>Founding member of Vanta's Venture &amp; Startup Partnerships team in EMEA. Build and scale presence across London startup and VC ecosystem.</t>
+        </is>
+      </c>
+      <c r="L30" s="8" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/vanta/4e32f84c-84c5-45a6-a8b5-2b3f71235286</t>
+        </is>
+      </c>
+      <c r="M30" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N30" s="8" t="inlineStr">
+        <is>
+          <t>Ashby</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Director BD matches VP seniority. Defense tech partially aligns. Air Dominance division is high-profile. UK pension plan (36/40 skills, 18/35 industry, 22/25 experience).</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Anduril Industries</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Director, Business Development - Mission Autonomy</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Defense Tech</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J31" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K31" s="10" t="inlineStr">
+        <is>
+          <t>Director BD within Air Dominance and Strike division. Identify, shape, capture, and grow new opportunities. UK &amp; IE pension plan included.</t>
+        </is>
+      </c>
+      <c r="L31" s="11" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/andurilindustries/jobs/5056776007</t>
+        </is>
+      </c>
+      <c r="M31" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N31" s="11" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="45" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>REPEAT</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n">
-        <v>76</v>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>CoS operator skills transfer to product context. Fintech sector fully aligns but product-specific focus less direct than CEO-facing roles (24/40 skills, 35/35 industry, 17/25 experience).</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Monzo</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Chief of Staff to CPO</t>
-        </is>
-      </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>Fintech/Banking</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="inlineStr">
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>BD at homebuying fintech. Financial services sector partially aligns. Regional scope manageable (32/40 skills, 28/35 industry, 16/25 experience).</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Gen H</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Business Development Manager (London &amp; South East)</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Fintech/Mortgage</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="H30" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I30" s="8" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J30" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K30" s="7" t="inlineStr">
-        <is>
-          <t>Chief of Staff to the Chief Product Officer. Support CPO and product leadership team in setting product vision and strategy for Monzo.</t>
-        </is>
-      </c>
-      <c r="L30" s="8" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/monzo/jobs/4589197</t>
-        </is>
-      </c>
-      <c r="M30" s="8" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N30" s="8" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="45" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B31" s="15" t="n">
-        <v>76</v>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>Director-level agency partnerships at martech platform. Strategy and execution for scaling agency ecosystem. London hub available (38/40 skills, 18/35 industry, 20/25 experience).</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>Attentive</t>
-        </is>
-      </c>
-      <c r="E31" s="11" t="inlineStr">
-        <is>
-          <t>Director - Partnerships (Agency Partners)</t>
-        </is>
-      </c>
-      <c r="F31" s="11" t="inlineStr">
-        <is>
-          <t>Martech/Communications</t>
-        </is>
-      </c>
-      <c r="G31" s="11" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
-      <c r="H31" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I31" s="11" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J31" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K31" s="10" t="inlineStr">
-        <is>
-          <t>Director of Agency Growth Partnerships, owning strategy and execution for scaling agency ecosystem. Employee hubs in New York City, San Francisco, London, and Sydney.</t>
-        </is>
-      </c>
-      <c r="L31" s="11" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/attentive/2a6e1948-6fbd-4f89-8bb5-12058a67eb02</t>
-        </is>
-      </c>
-      <c r="M31" s="11" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N31" s="11" t="inlineStr">
-        <is>
-          <t>Lever</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="45" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>REPEAT</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="n">
-        <v>75</v>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Excellent fintech sector fit at Monzo but CTO-facing role likely requires deeper technical background than Phil's commercial operator profile (20/40 skills, 35/35 industry, 20/25 experience).</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Monzo</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Chief of Staff - CTO</t>
-        </is>
-      </c>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>Fintech/Banking</t>
-        </is>
-      </c>
-      <c r="G32" s="8" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -2525,12 +2586,12 @@
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>Chief of Staff to CTO at Monzo. Work closely with leaders across engineering, data, and security functions (~700 people). London office at least once per week.</t>
+          <t>BD Manager at Gen H, rebuilding the homebuying process. Focused on London and South East region.</t>
         </is>
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/monzo/jobs/7019979</t>
+          <t>https://boards.greenhouse.io/generationhome/jobs/4279993101</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
@@ -2550,27 +2611,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B33" s="15" t="n">
-        <v>73</v>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Hard tech sector partially aligns with resume focus. Autonomous maritime systems are niche but BD skills transfer directly (30/40 skills, 25/35 industry, 18/25 experience).</t>
+          <t>CoS operator skills transfer to product context. Fintech sector fully aligns (24/40 skills, 35/35 industry, 17/25 experience).</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Saronic</t>
+          <t>Monzo</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>Business Development - London</t>
+          <t>Chief of Staff to the Chief Product Officer</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>Hard Tech/Defense</t>
+          <t>Fintech/Banking</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr">
@@ -2595,12 +2658,12 @@
       </c>
       <c r="K33" s="10" t="inlineStr">
         <is>
-          <t>Drive growth by identifying new opportunities, building customer partnerships, and expanding footprint in UK and EU. Autonomous maritime technology focus.</t>
+          <t>Report directly to CPO. Massive scope role leading product strategy for Monzo.</t>
         </is>
       </c>
       <c r="L33" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/saronic/1afc5730-44dd-412b-9f38-81484276b466</t>
+          <t>https://job-boards.greenhouse.io/monzo/jobs/5910266</t>
         </is>
       </c>
       <c r="M33" s="11" t="inlineStr">
@@ -2610,42 +2673,44 @@
       </c>
       <c r="N33" s="11" t="inlineStr">
         <is>
-          <t>Lever</t>
+          <t>Greenhouse</t>
         </is>
       </c>
     </row>
     <row r="34" ht="45" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>REPEAT</t>
-        </is>
-      </c>
-      <c r="B34" s="15" t="n">
-        <v>72</v>
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>CoS operator skills transfer to nonprofit context. Education/philanthropy sector less fintech-aligned but strong mission and DC hybrid location is excellent (32/40 skills, 15/35 industry, 25/25 experience).</t>
+          <t>News partnerships at OpenAI. AI sector strong. EMEA scope. Partnership management matches but news-specific (30/40 skills, 28/35 industry, 18/25 experience).</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Strada Education Foundation</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>Chief of Staff</t>
+          <t>Partner Manager, News - EMEA</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>Education/Nonprofit</t>
+          <t>AI/Technology</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>Washington DC</t>
+          <t>London</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr">
@@ -2665,12 +2730,12 @@
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>Trusted strategic partner to CEO. Enhance CEO effectiveness by strengthening organizational alignment, tackling special projects, accelerating priority initiatives. Senior Leadership Team member.</t>
+          <t>Build and nurture relationships with news publishing partners through 1:1 interactions and industry programs.</t>
         </is>
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/stradaeducation/6037a259-de9d-4733-a7f8-cbbb6f7d5bdd</t>
+          <t>https://jobs.ashbyhq.com/openai/77a2ec4a-10ee-4c7e-b05f-881348b9b41f</t>
         </is>
       </c>
       <c r="M34" s="8" t="inlineStr">
@@ -2680,7 +2745,7 @@
       </c>
       <c r="N34" s="8" t="inlineStr">
         <is>
-          <t>Lever</t>
+          <t>Ashby</t>
         </is>
       </c>
     </row>
@@ -2690,27 +2755,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B35" s="15" t="n">
-        <v>72</v>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>CoS operator skills transfer but health tech sector is outside Phil's fintech/banking core. VP-level role matches seniority (30/40 skills, 18/35 industry, 24/25 experience).</t>
+          <t>Excellent fintech sector fit but CTO-facing role requires deeper technical background (20/40 skills, 35/35 industry, 20/25 experience).</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Eucalyptus</t>
+          <t>Monzo</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>Chief of Staff (VP of Operations)</t>
+          <t>Chief of Staff - CTO</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>Health Tech</t>
+          <t>Fintech/Banking</t>
         </is>
       </c>
       <c r="G35" s="11" t="inlineStr">
@@ -2735,12 +2802,12 @@
       </c>
       <c r="K35" s="10" t="inlineStr">
         <is>
-          <t>Chief of Staff to VP of Operations. Lead mission-critical projects end-to-end, tackle complex problems, align cross-functional teams. London HQ.</t>
+          <t>CoS to CTO working with leaders across engineering, data, and security (~700 people).</t>
         </is>
       </c>
       <c r="L35" s="11" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/eucalyptus/jobs/4616727005</t>
+          <t>https://job-boards.greenhouse.io/monzo/jobs/7019979</t>
         </is>
       </c>
       <c r="M35" s="11" t="inlineStr">
@@ -2755,102 +2822,106 @@
       </c>
     </row>
     <row r="36" ht="45" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Defense/autonomy BD at Applied Intuition. DC location strong. Defense tech partially aligned (34/40 skills, 20/35 industry, 20/25 experience).</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Applied Intuition</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Business Development Growth Lead - Ground/Air Mission Autonomy</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Defense/Autonomy Tech</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>BD Growth Lead for Ground/Air Mission Autonomy. Driving growth in defense and autonomous systems.</t>
+        </is>
+      </c>
+      <c r="L36" s="8" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/appliedintuition/jobs/6547513002</t>
+        </is>
+      </c>
+      <c r="M36" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N36" s="8" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="45" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B36" s="15" t="n">
-        <v>72</v>
-      </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>Public financial management has partial alignment with banking background. BD leadership matches experience. Government sector less aligned (30/40 skills, 22/35 industry, 20/25 experience).</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>FreeBalance</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Business Development Manager</t>
-        </is>
-      </c>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>Gov Tech/Public Finance</t>
-        </is>
-      </c>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t>Washington DC</t>
-        </is>
-      </c>
-      <c r="H36" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I36" s="8" t="inlineStr">
-        <is>
-          <t>In-Office</t>
-        </is>
-      </c>
-      <c r="J36" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K36" s="7" t="inlineStr">
-        <is>
-          <t>Lead efforts to identify, manage and develop new business opportunities in the global Public Financial Management market. 5-7 years relevant experience required.</t>
-        </is>
-      </c>
-      <c r="L36" s="8" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/freebalance.com/0793ba14-5fc0-4608-8d4f-fc950ad4cb5c</t>
-        </is>
-      </c>
-      <c r="M36" s="8" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N36" s="8" t="inlineStr">
-        <is>
-          <t>Lever</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="45" customHeight="1">
-      <c r="A37" s="14" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="n">
-        <v>72</v>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Chief of Staff to CRO at martech platform. Strategy, operations, and program leadership blend. London hub available. 5-8+ years experience required (34/40 skills, 18/35 industry, 20/25 experience).</t>
+          <t>Partnership development skills transfer. Energy tech less aligned but financial services partnerships relevant (30/40 skills, 20/35 industry, 24/25 experience).</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>Attentive</t>
+          <t>Octopus Energy</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>Chief of Staff - CRO</t>
+          <t>Partnerships Manager</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>Martech/Communications</t>
+          <t>Energy Tech</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr">
@@ -2875,12 +2946,12 @@
       </c>
       <c r="K37" s="10" t="inlineStr">
         <is>
-          <t>Chief of Staff to the Chief Revenue Officer. Drive alignment, operating rigor, and execution across end-to-end Revenue organization. Attend weekly C-Level Executive meetings and quarterly Board Meetings.</t>
+          <t>Face and voice of Octopus Electric Vehicles across financial services and employee benefits.</t>
         </is>
       </c>
       <c r="L37" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/attentive/f470da25-9907-48a1-bb13-a300ab16ee4e</t>
+          <t>https://jobs.lever.co/octoenergy/2ca2854d-1dfa-4a02-9959-0346399d20bd</t>
         </is>
       </c>
       <c r="M37" s="11" t="inlineStr">
@@ -2900,242 +2971,250 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="B38" s="15" t="n">
-        <v>71</v>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Chief of Staff as close collaborator to executive team and right hand to CEO. Music/entertainment tech sector not fintech-aligned but iconic brand (34/40 skills, 15/35 industry, 22/25 experience).</t>
+          <t>VC partnerships at Deel matches Phil's VC background. HR/payroll unicorn. Remote-first (34/40 skills, 22/35 industry, 18/25 experience).</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>SoundCloud</t>
+          <t>Deel</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>Chief of Staff</t>
+          <t>Partnerships Manager, Venture Capital</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>Music/Entertainment Tech</t>
+          <t>HR Tech/Payroll</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
+          <t>Remote-Global</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>Remote-Global</t>
+        </is>
+      </c>
+      <c r="J38" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>Partnerships Manager in Venture Capital team at Deel, managing VC and startup ecosystem relationships.</t>
+        </is>
+      </c>
+      <c r="L38" s="8" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/deel/90aefa1d-30b5-4b43-82c2-53348fbc64b9</t>
+        </is>
+      </c>
+      <c r="M38" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N38" s="8" t="inlineStr">
+        <is>
+          <t>Ashby</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="45" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>Global remit partnerships management. Travel/mobility not fintech-aligned but strategic partnership development is direct match (35/40 skills, 15/35 industry, 23/25 experience).</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>Blacklane</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Lead Strategic Partnerships Manager</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>Mobility/Travel Tech</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
           <t>London</t>
         </is>
       </c>
-      <c r="H38" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I38" s="8" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J38" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K38" s="7" t="inlineStr">
-        <is>
-          <t>Serve as close collaborator to the executive team and right hand to the CEO, driving the CEO's most critical priorities. Offices in US, Germany, and UK (London).</t>
-        </is>
-      </c>
-      <c r="L38" s="8" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/soundcloud71/jobs/7743899002</t>
-        </is>
-      </c>
-      <c r="M38" s="8" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N38" s="8" t="inlineStr">
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J39" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K39" s="10" t="inlineStr">
+        <is>
+          <t>Drive business growth with global remit. Establish and nurture key partnerships.</t>
+        </is>
+      </c>
+      <c r="L39" s="11" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/blacklane/jobs/7789460002</t>
+        </is>
+      </c>
+      <c r="M39" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N39" s="11" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="45" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
+    <row r="40" ht="45" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Head of partnerships with P&amp;L ownership. PropTech/energy sector not fintech-aligned (36/40 skills, 15/35 industry, 22/25 experience).</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Goodlord</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Head of Partnerships - Energy</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>PropTech/Energy</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>Remote-Global</t>
+        </is>
+      </c>
+      <c r="J40" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>Own single strategic OVO Energy partnership. Lead small team of 3 ICs.</t>
+        </is>
+      </c>
+      <c r="L40" s="8" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/goodlord/125cc074-38d8-4d5d-ada1-03392e4ef7ac</t>
+        </is>
+      </c>
+      <c r="M40" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N40" s="8" t="inlineStr">
+        <is>
+          <t>Ashby</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="45" customHeight="1">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="B39" s="15" t="n">
-        <v>71</v>
-      </c>
-      <c r="C39" s="10" t="inlineStr">
-        <is>
-          <t>Chief of Staff to Global Chief People Officer at WPP. Requires 12+ years experience. Visionary enterprise-minded leader. London headquarters (34/40 skills, 15/35 industry, 22/25 experience).</t>
-        </is>
-      </c>
-      <c r="D39" s="11" t="inlineStr">
-        <is>
-          <t>WPP</t>
-        </is>
-      </c>
-      <c r="E39" s="11" t="inlineStr">
-        <is>
-          <t>Chief of Staff to Global CPO</t>
-        </is>
-      </c>
-      <c r="F39" s="11" t="inlineStr">
-        <is>
-          <t>Advertising/Media</t>
-        </is>
-      </c>
-      <c r="G39" s="11" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
-      <c r="H39" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I39" s="11" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J39" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K39" s="10" t="inlineStr">
-        <is>
-          <t>Chief of Staff to the Global Chief People Officer at WPP. Requires 12+ years in strategy, transformation or Chief of Staff roles in global, matrixed organisations. London/Singapore/New York.</t>
-        </is>
-      </c>
-      <c r="L39" s="11" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/wpp/jobs/8364683002</t>
-        </is>
-      </c>
-      <c r="M39" s="11" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N39" s="11" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="45" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B40" s="15" t="n">
-        <v>71</v>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>Business Development Manager at mortgage tech startup. BD role matches commercial background. Housing/mortgage tech adjacent to fintech (30/40 skills, 25/35 industry, 16/25 experience).</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Gen H</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Business Development Manager - London &amp; South East</t>
-        </is>
-      </c>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>Mortgage Tech/Fintech</t>
-        </is>
-      </c>
-      <c r="G40" s="8" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
-      <c r="H40" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I40" s="8" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J40" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K40" s="7" t="inlineStr">
-        <is>
-          <t>Business Development Manager focused on London &amp; South East region. Gen H is rebuilding the homebuying process to make it simple, transparent and fair.</t>
-        </is>
-      </c>
-      <c r="L40" s="8" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/generationhome/jobs/4279993101</t>
-        </is>
-      </c>
-      <c r="M40" s="8" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N40" s="8" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="45" customHeight="1">
-      <c r="A41" s="9" t="inlineStr">
-        <is>
-          <t>REPEAT</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="n">
-        <v>70</v>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>Partnership development skills transfer. Sports tech sector is not aligned with Phil's fintech core but strong brand and Strava backing add appeal (30/40 skills, 15/35 industry, 25/25 experience).</t>
+          <t>VP of partnerships at civic tech. DC likely location. Government sector less aligned but partnerships match (36/40 skills, 15/35 industry, 22/25 experience).</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Runna</t>
+          <t>CivicMarketplace</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>Partnerships Lead - UK</t>
+          <t>VP of Partnerships</t>
         </is>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>Sports Tech</t>
+          <t>GovTech/Civic</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Washington DC</t>
         </is>
       </c>
       <c r="H41" s="11" t="inlineStr">
@@ -3155,12 +3234,12 @@
       </c>
       <c r="K41" s="10" t="inlineStr">
         <is>
-          <t>Lead UK partnerships for Runna, the #1 training platform for runners. Apple iPhone app of the year finalist, acquired by Strava in 2025.</t>
+          <t>Build trusted relationships with associations and local government leaders. Turn opportunities into impact and revenue.</t>
         </is>
       </c>
       <c r="L41" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/runna/30ace097-9621-40cd-904d-59fe6359d50b</t>
+          <t>https://jobs.ashbyhq.com/civicmarketplace/1a1b5b1f-b702-4e62-927a-b6030205b371</t>
         </is>
       </c>
       <c r="M41" s="11" t="inlineStr">
@@ -3180,27 +3259,29 @@
           <t>REPEAT</t>
         </is>
       </c>
-      <c r="B42" s="15" t="n">
-        <v>70</v>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>BD skills transfer but role level (2+ years) is significantly below Phil's VP experience. SaaS/marketplace sector partially relevant (25/40 skills, 20/35 industry, 25/25 experience).</t>
+          <t>CoS operator skills transfer but health tech outside fintech core (30/40 skills, 18/35 industry, 24/25 experience).</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>Fresha</t>
+          <t>Eucalyptus</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Business Development Manager - London</t>
+          <t>Chief of Staff (VP of Operations)</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>SaaS/Marketplace</t>
+          <t>Health Tech</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
@@ -3215,46 +3296,766 @@
       </c>
       <c r="I42" s="8" t="inlineStr">
         <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J42" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>CoS to VP of Operations. Lead mission-critical projects, tackle complex problems.</t>
+        </is>
+      </c>
+      <c r="L42" s="8" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/eucalyptus/jobs/4616727005</t>
+        </is>
+      </c>
+      <c r="M42" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N42" s="8" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>CoS operator skills transfer to nonprofit context. DC hybrid with CEO is excellent (32/40 skills, 15/35 industry, 25/25 experience).</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>Strada Education Foundation</t>
+        </is>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>Chief of Staff</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>Education/Nonprofit</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I43" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J43" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K43" s="10" t="inlineStr">
+        <is>
+          <t>Trusted strategic partner to CEO. Enhance CEO effectiveness, strengthen alignment, tackle special projects.</t>
+        </is>
+      </c>
+      <c r="L43" s="11" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/stradaeducation/6037a259-de9d-4733-a7f8-cbbb6f7d5bdd</t>
+        </is>
+      </c>
+      <c r="M43" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N43" s="11" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="45" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>CoS to CRO with strategy, operations, program leadership. Martech/communications adjacent. London hub. 5-8+ years (34/40 skills, 18/35 industry, 20/25 experience).</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Attentive</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Chief of Staff - CRO</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>Martech/Communications</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J44" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>CoS to CRO driving alignment, rigor, execution across Revenue org. 5-8+ years required.</t>
+        </is>
+      </c>
+      <c r="L44" s="8" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/attentive/f470da25-9907-48a1-bb13-a300ab16ee4e</t>
+        </is>
+      </c>
+      <c r="M44" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N44" s="8" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="45" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>Strategic partnerships focus matches expertise. Policy/advocacy less fintech-aligned but Arlington VA near DC (35/40 skills, 15/35 industry, 22/25 experience).</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>Stand Together</t>
+        </is>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>Strategic Partnerships Manager</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>Policy/Advocacy</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>Arlington VA</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I45" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J45" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K45" s="10" t="inlineStr">
+        <is>
+          <t>Strategy development and execution of coalition efforts. Leverage relationships for federal outcomes.</t>
+        </is>
+      </c>
+      <c r="L45" s="11" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/standtogether/c3c9ed59-ce89-44a2-aedc-bad9f7226705</t>
+        </is>
+      </c>
+      <c r="M45" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N45" s="11" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="45" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Public financial management has partial alignment. BD leadership matches experience (30/40 skills, 22/35 industry, 20/25 experience).</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>FreeBalance</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Business Development Manager</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Gov Tech/Public Finance</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I46" s="8" t="inlineStr">
+        <is>
           <t>In-Office</t>
         </is>
       </c>
-      <c r="J42" s="8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K42" s="7" t="inlineStr">
-        <is>
-          <t>100% focused on bringing in new business development. London HQ at The Bower, Old Street. Requires 2+ years B2B sales experience in SaaS, marketplaces, or payments.</t>
-        </is>
-      </c>
-      <c r="L42" s="8" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/fresha/ca5ccd83-1c6d-46d8-839f-db6958e79924</t>
-        </is>
-      </c>
-      <c r="M42" s="8" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N42" s="8" t="inlineStr">
+      <c r="J46" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t>Lead BD efforts in global Public Financial Management market. 5-7 years relevant experience.</t>
+        </is>
+      </c>
+      <c r="L46" s="8" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/freebalance.com/0793ba14-5fc0-4608-8d4f-fc950ad4cb5c</t>
+        </is>
+      </c>
+      <c r="M46" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N46" s="8" t="inlineStr">
         <is>
           <t>Lever</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+    <row r="47" ht="45" customHeight="1">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>Defense/maritime BD in London. Strong seniority match. Defense tech partially aligned (34/40 skills, 18/35 industry, 20/25 experience).</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>Saronic Technologies</t>
+        </is>
+      </c>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>Business Development - London</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>Defense/Maritime Tech</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I47" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J47" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K47" s="10" t="inlineStr">
+        <is>
+          <t>Drive growth by identifying new opportunities in UK and EU. Proven experience in defense, maritime, or technology BD.</t>
+        </is>
+      </c>
+      <c r="L47" s="11" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/saronic/1afc5730-44dd-412b-9f38-81484276b466</t>
+        </is>
+      </c>
+      <c r="M47" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N47" s="11" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="45" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>CoS operator skills transfer but edtech outside fintech core (30/40 skills, 15/35 industry, 25/25 experience).</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Zen Educate</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Chief of Staff</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>EdTech</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I48" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J48" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>CoS at edtech startup. Zero-to-one company-building opportunity.</t>
+        </is>
+      </c>
+      <c r="L48" s="8" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/zeneducate/957cc2f0-49d7-484b-9fad-a34ee78b64bb</t>
+        </is>
+      </c>
+      <c r="M48" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N48" s="8" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="45" customHeight="1">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>Banking infrastructure strategic partnerships. Fintech perfectly aligned but likely SF/NYC-based (36/40 skills, 35/35 industry, 0/25 experience - location uncertain).</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>Strategic Partnerships Lead</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>Fintech/Banking Infrastructure</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="H49" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J49" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K49" s="10" t="inlineStr">
+        <is>
+          <t>Strategic Partnerships Lead at Column, a bank and software company built from the ground up for builders.</t>
+        </is>
+      </c>
+      <c r="L49" s="11" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/column/83c71171-e327-45e2-8b58-cfe5ee16209a</t>
+        </is>
+      </c>
+      <c r="M49" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N49" s="11" t="inlineStr">
+        <is>
+          <t>Ashby</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="45" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>CoS operator skills transfer. Agriculture/nonprofit sector far from fintech core (32/40 skills, 12/35 industry, 25/25 experience).</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>One Acre Fund</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Chief of Staff to the President</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>Agriculture/Nonprofit</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>Remote-US</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I50" s="8" t="inlineStr">
+        <is>
+          <t>Remote-US</t>
+        </is>
+      </c>
+      <c r="J50" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>Work closely with the President. Preference for US East Coast cities including DC.</t>
+        </is>
+      </c>
+      <c r="L50" s="8" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/oneacrefundglobal/jobs/7587830</t>
+        </is>
+      </c>
+      <c r="M50" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N50" s="8" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="45" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>Strategic/operational partner to CSO. Healthcare sector not fintech-aligned but DC location strong (32/40 skills, 16/35 industry, 22/25 experience).</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>Aledade</t>
+        </is>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>Chief of Staff, Strategy</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>Healthcare/Value-Based Care</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="H51" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I51" s="11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J51" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K51" s="10" t="inlineStr">
+        <is>
+          <t>Strategic and operational partner to Chief Strategy Officer. 10+ years professional experience required.</t>
+        </is>
+      </c>
+      <c r="L51" s="11" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/aledade/2cf2e14f-9f7d-483a-a80f-55dccd959389</t>
+        </is>
+      </c>
+      <c r="M51" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N51" s="11" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="45" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>REPEAT</t>
+        </is>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Partnership development skills transfer. Sports tech not aligned with fintech core (30/40 skills, 15/35 industry, 25/25 experience).</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Runna</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Partnerships Lead - UK</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>Sports Tech</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="H52" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I52" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J52" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr">
+        <is>
+          <t>Lead UK partnerships for Runna, #1 training platform for runners. Acquired by Strava.</t>
+        </is>
+      </c>
+      <c r="L52" s="8" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/runna/30ace097-9621-40cd-904d-59fe6359d50b</t>
+        </is>
+      </c>
+      <c r="M52" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N52" s="8" t="inlineStr">
+        <is>
+          <t>Ashby</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
         <is>
           <t>Score Key: 🟢 90+ Elite | 🔵 80-89 Strong | 🟡 70-79 Good | 🔴 Below 70</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:N42"/>
+  <autoFilter ref="A5:N52"/>
   <mergeCells count="4">
-    <mergeCell ref="A45:N45"/>
+    <mergeCell ref="A55:N55"/>
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>